<commit_message>
Pruebas finales de destajista y mandos intermedios terminadas
</commit_message>
<xml_diff>
--- a/data/CONCEPTOS BD.xlsx
+++ b/data/CONCEPTOS BD.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\DESTAJOS FLET\Base de datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\DESTAJOS FLET\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664DF994-DEFB-4FCF-A6EC-5E5E0A94793C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842EB9EB-9E31-4243-B7AB-733D090BCBCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E3DEF130-6E41-43F9-9115-ADD929837210}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="1386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2638" uniqueCount="1626">
   <si>
     <t>ABB01</t>
   </si>
@@ -4202,16 +4202,737 @@
   </si>
   <si>
     <t>clave</t>
+  </si>
+  <si>
+    <t>TACEITE</t>
+  </si>
+  <si>
+    <t>Limpiar y aplicar aceite o barniz sobre madera</t>
+  </si>
+  <si>
+    <t>TALB</t>
+  </si>
+  <si>
+    <t>Albañil por el día</t>
+  </si>
+  <si>
+    <t>TALJIBE</t>
+  </si>
+  <si>
+    <t>Aljibe de block, incluye armado, cimbra, colado dalas ,castillos,zarpeo y enjarre</t>
+  </si>
+  <si>
+    <t>TARMC</t>
+  </si>
+  <si>
+    <t>Armado de castillo con varilla de 3/8" y estribos alambrón @ 20 cms</t>
+  </si>
+  <si>
+    <t>TBANCOC</t>
+  </si>
+  <si>
+    <t>Banquetón de cocina pulido</t>
+  </si>
+  <si>
+    <t>TBODEGA</t>
+  </si>
+  <si>
+    <t>Armar bodega y baño con fajillas y malla en exterior, colocar puertas</t>
+  </si>
+  <si>
+    <t>TBOQ</t>
+  </si>
+  <si>
+    <t>Boquilla en puertas y ventanas</t>
+  </si>
+  <si>
+    <t>TBOV</t>
+  </si>
+  <si>
+    <t>Instalar bóveda de cuña en sucio en vigas de acero</t>
+  </si>
+  <si>
+    <t>TCCASO</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar castillo de soga</t>
+  </si>
+  <si>
+    <t>TCCASO3</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar castillo de soga 3 caras</t>
+  </si>
+  <si>
+    <t>TCCATE</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar castillo de tezón</t>
+  </si>
+  <si>
+    <t>TCCATE3</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar castillo de tezón 3 caras</t>
+  </si>
+  <si>
+    <t>TCCESO</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar cerramiento de soga</t>
+  </si>
+  <si>
+    <t>TCCETE</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar cerramiento de tezón</t>
+  </si>
+  <si>
+    <t>TCDASO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armar, cimbrar y colar dala de 15 x 20 </t>
+  </si>
+  <si>
+    <t>TCDATE</t>
+  </si>
+  <si>
+    <t>Cimbrar y colar dala tezón con doble armex</t>
+  </si>
+  <si>
+    <t>TCENRAJ</t>
+  </si>
+  <si>
+    <t>Instalación de piso de rajuela a canto en cenefa ancho hasta 60 cms</t>
+  </si>
+  <si>
+    <t>TDADO</t>
+  </si>
+  <si>
+    <t>Colado de dado completo de 80x 80 x 80</t>
+  </si>
+  <si>
+    <t>TENJADO</t>
+  </si>
+  <si>
+    <t>Zarpeo, enjarre y figurado tipo adobe con estrías</t>
+  </si>
+  <si>
+    <t>TENJAFB</t>
+  </si>
+  <si>
+    <t>Enjarre en bóveda terminado afinado, incluye andamios</t>
+  </si>
+  <si>
+    <t>TENJAFM</t>
+  </si>
+  <si>
+    <t>Enjarre en muro terminado afinado, incluye andamios</t>
+  </si>
+  <si>
+    <t>TENJAP</t>
+  </si>
+  <si>
+    <t>Enjarre en muro terminado apalillado, incluye andamios</t>
+  </si>
+  <si>
+    <t>TENJB</t>
+  </si>
+  <si>
+    <t>Enjarre en bóveda, incluye zarpeos y andamios</t>
+  </si>
+  <si>
+    <t>TENJCP</t>
+  </si>
+  <si>
+    <t>Enjarre a tallón de cuchara pulido</t>
+  </si>
+  <si>
+    <t>TEXCAV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excavación terreno </t>
+  </si>
+  <si>
+    <t>TFILTRO</t>
+  </si>
+  <si>
+    <t>Filtro de grava de 10 cms compactada</t>
+  </si>
+  <si>
+    <t>TFIRJAL</t>
+  </si>
+  <si>
+    <t>Colocar jal con malla electro-soldada y lechadeado</t>
+  </si>
+  <si>
+    <t>TFOSA</t>
+  </si>
+  <si>
+    <t>Excavación, forjado y terminado de fosa séptica con filtros</t>
+  </si>
+  <si>
+    <t>TIMP</t>
+  </si>
+  <si>
+    <t>Raspado de superficie, repellado e impermeabilizado azotea</t>
+  </si>
+  <si>
+    <t>TJALIN</t>
+  </si>
+  <si>
+    <t>Colocar jal en techo inclinado, incluye malla y apalillado</t>
+  </si>
+  <si>
+    <t>TJALP</t>
+  </si>
+  <si>
+    <t>Colocar jal en techo plano, incluye malla y apalillado</t>
+  </si>
+  <si>
+    <t>TLADAZ</t>
+  </si>
+  <si>
+    <t>Instalar ladrillo de azotea sobre superficies de azotea, incluye acarreos</t>
+  </si>
+  <si>
+    <t>TLADAZA</t>
+  </si>
+  <si>
+    <t>Colocar piso de barro y juntear, detallar y limpiar terminado aparente</t>
+  </si>
+  <si>
+    <t>TLODADOB</t>
+  </si>
+  <si>
+    <t>Aplicar sellador y lodo sobre superficie de adobe terminado</t>
+  </si>
+  <si>
+    <t>TLOSA</t>
+  </si>
+  <si>
+    <t>Colocar malla, colado de losa concreto y repellado</t>
+  </si>
+  <si>
+    <t>TLOSDESP</t>
+  </si>
+  <si>
+    <t>Trazo, ranuras, barrenos, armar, cimbrar y colar losa despensa terminado</t>
+  </si>
+  <si>
+    <t>TMAM1R40</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 1 rostro de 40 cms</t>
+  </si>
+  <si>
+    <t>TMAM1R40jc</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 1 rostro de 40 cms junta cerrada</t>
+  </si>
+  <si>
+    <t>TMAM1R50</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 1 rostro de 50 cms</t>
+  </si>
+  <si>
+    <t>TMAM1R60</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 1 rostro de 60 cms</t>
+  </si>
+  <si>
+    <t>TMAM2R</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 2 rostros de 40 a 50 cms</t>
+  </si>
+  <si>
+    <t>TMAM2R40</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 2 rostros de 40 cms</t>
+  </si>
+  <si>
+    <t>TMAM2R50</t>
+  </si>
+  <si>
+    <t>Mamposteo de piedra 2 rostros de 50 cms</t>
+  </si>
+  <si>
+    <t>TMCAP</t>
+  </si>
+  <si>
+    <t>Muro de capuchino en sucio</t>
+  </si>
+  <si>
+    <t>TMOCSO</t>
+  </si>
+  <si>
+    <t>Mocheta de soga en sucio</t>
+  </si>
+  <si>
+    <t>TMOCTE</t>
+  </si>
+  <si>
+    <t>Mocheta de tezón en sucio</t>
+  </si>
+  <si>
+    <t>TMSOG</t>
+  </si>
+  <si>
+    <t>Muro de soga en sucio</t>
+  </si>
+  <si>
+    <t>TMTEZ</t>
+  </si>
+  <si>
+    <t>Muro de tezón en sucio</t>
+  </si>
+  <si>
+    <t>TMUADOSO</t>
+  </si>
+  <si>
+    <t>Muro de adobe de soga en sucio no importa altura, inlcuye junta</t>
+  </si>
+  <si>
+    <t>TMUADOTE</t>
+  </si>
+  <si>
+    <t>TNIVMR</t>
+  </si>
+  <si>
+    <t>Nivelación de muro de piedra con rostro</t>
+  </si>
+  <si>
+    <t>TPEO</t>
+  </si>
+  <si>
+    <t>Peón por el día</t>
+  </si>
+  <si>
+    <t>TPINT</t>
+  </si>
+  <si>
+    <t>Raspar, resanes, sellador y pintura terminado sobre muros y bóvedas</t>
+  </si>
+  <si>
+    <t>TPISO</t>
+  </si>
+  <si>
+    <t>Lechadeo, colocar malla, colado de piso repellado</t>
+  </si>
+  <si>
+    <t>TPISORAJ</t>
+  </si>
+  <si>
+    <t>Instalación de piso de rajuela a canto en pisos</t>
+  </si>
+  <si>
+    <t>TREG</t>
+  </si>
+  <si>
+    <t>Excavación, forjado y terminado registro sanitario 1.00x1.00x1.00</t>
+  </si>
+  <si>
+    <t>TRELLM</t>
+  </si>
+  <si>
+    <t>Relleno y compactación en capas de 20 cms con apoyo de máquina</t>
+  </si>
+  <si>
+    <t>TREN</t>
+  </si>
+  <si>
+    <t>Renchido de piedra</t>
+  </si>
+  <si>
+    <t>TSUBVIGA</t>
+  </si>
+  <si>
+    <t>subir y nivelar cerramientos de madera ( incluye fester, resanes y colados )</t>
+  </si>
+  <si>
+    <t>TTEJA</t>
+  </si>
+  <si>
+    <t>Tejar, inculye costuras y caballeteros</t>
+  </si>
+  <si>
+    <t>TVADO</t>
+  </si>
+  <si>
+    <t>Vado pluvial de 1 metro de ancho</t>
+  </si>
+  <si>
+    <t>SJABB01</t>
+  </si>
+  <si>
+    <t>SJABB02</t>
+  </si>
+  <si>
+    <t>SJABB03</t>
+  </si>
+  <si>
+    <t>SJABB05</t>
+  </si>
+  <si>
+    <t>SJABB06</t>
+  </si>
+  <si>
+    <t>SJABB07</t>
+  </si>
+  <si>
+    <t>SJAFI01</t>
+  </si>
+  <si>
+    <t>SJAFI02</t>
+  </si>
+  <si>
+    <t>SJAFI03</t>
+  </si>
+  <si>
+    <t>SJAFIEX</t>
+  </si>
+  <si>
+    <t>SJANC02</t>
+  </si>
+  <si>
+    <t>SJANC03</t>
+  </si>
+  <si>
+    <t>SJARM01</t>
+  </si>
+  <si>
+    <t>SJARM04</t>
+  </si>
+  <si>
+    <t>SJARM06</t>
+  </si>
+  <si>
+    <t>SJARM07</t>
+  </si>
+  <si>
+    <t>SJARM09</t>
+  </si>
+  <si>
+    <t>SJARM09A</t>
+  </si>
+  <si>
+    <t>SJARMTL</t>
+  </si>
+  <si>
+    <t>SJARMEX</t>
+  </si>
+  <si>
+    <t>SJBOQ02</t>
+  </si>
+  <si>
+    <t>SJBOQ06</t>
+  </si>
+  <si>
+    <t>SJBOQAF</t>
+  </si>
+  <si>
+    <t>SJCCA01</t>
+  </si>
+  <si>
+    <t>SJCCA02</t>
+  </si>
+  <si>
+    <t>SJCCA13</t>
+  </si>
+  <si>
+    <t>SJCCA14</t>
+  </si>
+  <si>
+    <t>SJCCA15</t>
+  </si>
+  <si>
+    <t>SJCCA16</t>
+  </si>
+  <si>
+    <t>SJCCA17</t>
+  </si>
+  <si>
+    <t>SJCDA07</t>
+  </si>
+  <si>
+    <t>SJCDA08</t>
+  </si>
+  <si>
+    <t>SJCCE20</t>
+  </si>
+  <si>
+    <t>SJCCE25</t>
+  </si>
+  <si>
+    <t>SJCCE35</t>
+  </si>
+  <si>
+    <t>SJCCECA</t>
+  </si>
+  <si>
+    <t>SJCCESO</t>
+  </si>
+  <si>
+    <t>SJCCETE</t>
+  </si>
+  <si>
+    <t>SJCIM04</t>
+  </si>
+  <si>
+    <t>SJCIM05</t>
+  </si>
+  <si>
+    <t>SJCOM01</t>
+  </si>
+  <si>
+    <t>SJCOM02</t>
+  </si>
+  <si>
+    <t>SJCONT1</t>
+  </si>
+  <si>
+    <t>SJENJ01</t>
+  </si>
+  <si>
+    <t>SJENJ02</t>
+  </si>
+  <si>
+    <t>SJENJ03</t>
+  </si>
+  <si>
+    <t>SJENJ04</t>
+  </si>
+  <si>
+    <t>SJENJ05</t>
+  </si>
+  <si>
+    <t>SJENJ07</t>
+  </si>
+  <si>
+    <t>SJENJ08</t>
+  </si>
+  <si>
+    <t>SJENJ09</t>
+  </si>
+  <si>
+    <t>SJEXC03</t>
+  </si>
+  <si>
+    <t>SJEXC04</t>
+  </si>
+  <si>
+    <t>SJFIR01</t>
+  </si>
+  <si>
+    <t>SJFIR02</t>
+  </si>
+  <si>
+    <t>SJGOT02</t>
+  </si>
+  <si>
+    <t>SJHOR01</t>
+  </si>
+  <si>
+    <t>SJHOR02</t>
+  </si>
+  <si>
+    <t>SJIMP01</t>
+  </si>
+  <si>
+    <t>SJIMP02</t>
+  </si>
+  <si>
+    <t>SJIMP03</t>
+  </si>
+  <si>
+    <t>SJMAM01</t>
+  </si>
+  <si>
+    <t>SJMAM02</t>
+  </si>
+  <si>
+    <t>SJMAM05</t>
+  </si>
+  <si>
+    <t>SJMBO05</t>
+  </si>
+  <si>
+    <t>SJMBO06</t>
+  </si>
+  <si>
+    <t>SJMBO07</t>
+  </si>
+  <si>
+    <t>SJMBO08</t>
+  </si>
+  <si>
+    <t>SJMSO1</t>
+  </si>
+  <si>
+    <t>SJMSO2</t>
+  </si>
+  <si>
+    <t>SJMTEZ1</t>
+  </si>
+  <si>
+    <t>SJMTEZ2</t>
+  </si>
+  <si>
+    <t>SJPER03</t>
+  </si>
+  <si>
+    <t>SJPIN01</t>
+  </si>
+  <si>
+    <t>SJPIN02</t>
+  </si>
+  <si>
+    <t>SJPIS08</t>
+  </si>
+  <si>
+    <t>SJPIS7</t>
+  </si>
+  <si>
+    <t>SJPIS72</t>
+  </si>
+  <si>
+    <t>SJPLA7</t>
+  </si>
+  <si>
+    <t>SJPOZO</t>
+  </si>
+  <si>
+    <t>SJPRE20</t>
+  </si>
+  <si>
+    <t>SJPRESO</t>
+  </si>
+  <si>
+    <t>SJPRETE</t>
+  </si>
+  <si>
+    <t>SJREC05</t>
+  </si>
+  <si>
+    <t>SJREC06</t>
+  </si>
+  <si>
+    <t>SJREC07</t>
+  </si>
+  <si>
+    <t>SJREC08</t>
+  </si>
+  <si>
+    <t>SJREC09</t>
+  </si>
+  <si>
+    <t>SJREG01</t>
+  </si>
+  <si>
+    <t>SJREG02</t>
+  </si>
+  <si>
+    <t>SJRELL03</t>
+  </si>
+  <si>
+    <t>SJRELL04</t>
+  </si>
+  <si>
+    <t>SJRELL05</t>
+  </si>
+  <si>
+    <t>SJRELLZAP</t>
+  </si>
+  <si>
+    <t>SJREN01</t>
+  </si>
+  <si>
+    <t>SJREN02</t>
+  </si>
+  <si>
+    <t>SJRES01</t>
+  </si>
+  <si>
+    <t>SJRESUMA1</t>
+  </si>
+  <si>
+    <t>Relleno de zanjas o zapatas suelo-cal /cemento con apoyo máquina</t>
+  </si>
+  <si>
+    <t>SJZAR02</t>
+  </si>
+  <si>
+    <t>Zarpeo de boveda</t>
+  </si>
+  <si>
+    <t>SJZAR03</t>
+  </si>
+  <si>
+    <t>Zarpeo de dalas y castillos</t>
+  </si>
+  <si>
+    <t>SJZAR04</t>
+  </si>
+  <si>
+    <t>Zarpeo de muro con cemento</t>
+  </si>
+  <si>
+    <t>SJZAR04f</t>
+  </si>
+  <si>
+    <t>Zarpeo de muro con manoseo para cubrir porocidad</t>
+  </si>
+  <si>
+    <t>SJTAP01</t>
+  </si>
+  <si>
+    <t>SJTAP02</t>
+  </si>
+  <si>
+    <t>SJTELA1</t>
+  </si>
+  <si>
+    <t>SJTELA2</t>
+  </si>
+  <si>
+    <t>SJTELA3</t>
+  </si>
+  <si>
+    <t>SJTRA01</t>
+  </si>
+  <si>
+    <t>SJTRA02</t>
+  </si>
+  <si>
+    <t>SJTRA03</t>
+  </si>
+  <si>
+    <t>acarreo y relleno con piedra braza acomodada para filtro base de cimentación</t>
+  </si>
+  <si>
+    <t>SJZAV01</t>
+  </si>
+  <si>
+    <t>SJZAV02</t>
+  </si>
+  <si>
+    <t>SJZAV03</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0&quot;.-&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="8"/>
       <name val="Arial"/>
@@ -4245,6 +4966,10 @@
       <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -4296,10 +5021,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4331,8 +5057,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -4635,7 +5368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1345250-224D-411D-A744-3FBD3D9C72D7}">
-  <dimension ref="A1:L705"/>
+  <dimension ref="A1:L879"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
@@ -20150,6 +20883,2442 @@
       <c r="K705" s="6"/>
       <c r="L705" s="6"/>
     </row>
+    <row r="706" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A706" s="1" t="s">
+        <v>1386</v>
+      </c>
+      <c r="B706" s="6" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C706" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D706" s="14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="707" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A707" s="1" t="s">
+        <v>1388</v>
+      </c>
+      <c r="B707" s="6" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C707" s="13" t="s">
+        <v>521</v>
+      </c>
+      <c r="D707" s="14">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="708" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A708" s="1" t="s">
+        <v>1390</v>
+      </c>
+      <c r="B708" s="6" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C708" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D708" s="14">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="709" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A709" s="1" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B709" s="6" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C709" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D709" s="14">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="710" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A710" s="1" t="s">
+        <v>1394</v>
+      </c>
+      <c r="B710" s="6" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C710" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D710" s="14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="711" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A711" s="1" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B711" s="6" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C711" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D711" s="14">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="712" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A712" s="1" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B712" s="6" t="s">
+        <v>1399</v>
+      </c>
+      <c r="C712" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D712" s="14">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="713" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A713" s="1" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B713" s="6" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C713" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D713" s="14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="714" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A714" s="1" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B714" s="6" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C714" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D714" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="715" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A715" s="1" t="s">
+        <v>1404</v>
+      </c>
+      <c r="B715" s="6" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C715" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D715" s="14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="716" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A716" s="1" t="s">
+        <v>1406</v>
+      </c>
+      <c r="B716" s="6" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C716" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D716" s="14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="717" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A717" s="1" t="s">
+        <v>1408</v>
+      </c>
+      <c r="B717" s="6" t="s">
+        <v>1409</v>
+      </c>
+      <c r="C717" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D717" s="14">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="718" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A718" s="1" t="s">
+        <v>1410</v>
+      </c>
+      <c r="B718" s="6" t="s">
+        <v>1411</v>
+      </c>
+      <c r="C718" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D718" s="14">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="719" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A719" s="1" t="s">
+        <v>1412</v>
+      </c>
+      <c r="B719" s="6" t="s">
+        <v>1413</v>
+      </c>
+      <c r="C719" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D719" s="14">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="720" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A720" s="1" t="s">
+        <v>1414</v>
+      </c>
+      <c r="B720" s="6" t="s">
+        <v>1415</v>
+      </c>
+      <c r="C720" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D720" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="721" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A721" s="1" t="s">
+        <v>1416</v>
+      </c>
+      <c r="B721" s="6" t="s">
+        <v>1417</v>
+      </c>
+      <c r="C721" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D721" s="14">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="722" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A722" s="1" t="s">
+        <v>1418</v>
+      </c>
+      <c r="B722" s="6" t="s">
+        <v>1419</v>
+      </c>
+      <c r="C722" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D722" s="14">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="723" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A723" s="1" t="s">
+        <v>1420</v>
+      </c>
+      <c r="B723" s="6" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C723" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D723" s="14">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="724" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A724" s="1" t="s">
+        <v>1422</v>
+      </c>
+      <c r="B724" s="6" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C724" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D724" s="14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="725" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A725" s="1" t="s">
+        <v>1424</v>
+      </c>
+      <c r="B725" s="6" t="s">
+        <v>1425</v>
+      </c>
+      <c r="C725" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D725" s="14">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="726" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A726" s="1" t="s">
+        <v>1426</v>
+      </c>
+      <c r="B726" s="6" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C726" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D726" s="14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="727" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A727" s="1" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B727" s="6" t="s">
+        <v>1429</v>
+      </c>
+      <c r="C727" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D727" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="728" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A728" s="1" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B728" s="6" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C728" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D728" s="14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="729" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A729" s="1" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B729" s="6" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C729" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D729" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="730" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A730" s="1" t="s">
+        <v>1434</v>
+      </c>
+      <c r="B730" s="6" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C730" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D730" s="14">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="731" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A731" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="B731" s="6" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C731" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D731" s="14">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="732" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A732" s="1" t="s">
+        <v>1438</v>
+      </c>
+      <c r="B732" s="6" t="s">
+        <v>1439</v>
+      </c>
+      <c r="C732" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D732" s="14">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="733" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A733" s="1" t="s">
+        <v>1440</v>
+      </c>
+      <c r="B733" s="6" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C733" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D733" s="14">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="734" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A734" s="1" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B734" s="6" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C734" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D734" s="14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="735" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A735" s="1" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B735" s="6" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C735" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D735" s="14">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="736" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A736" s="1" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B736" s="6" t="s">
+        <v>1447</v>
+      </c>
+      <c r="C736" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D736" s="14">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="737" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A737" s="1" t="s">
+        <v>1448</v>
+      </c>
+      <c r="B737" s="6" t="s">
+        <v>1449</v>
+      </c>
+      <c r="C737" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D737" s="14">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="738" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A738" s="1" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B738" s="6" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C738" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D738" s="14">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="739" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A739" s="1" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B739" s="6" t="s">
+        <v>1453</v>
+      </c>
+      <c r="C739" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D739" s="14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="740" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A740" s="1" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B740" s="6" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C740" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D740" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="741" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A741" s="1" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B741" s="6" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C741" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D741" s="14">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="742" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A742" s="1" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B742" s="6" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C742" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D742" s="14">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="743" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A743" s="1" t="s">
+        <v>1460</v>
+      </c>
+      <c r="B743" s="6" t="s">
+        <v>1461</v>
+      </c>
+      <c r="C743" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D743" s="14">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="744" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A744" s="1" t="s">
+        <v>1462</v>
+      </c>
+      <c r="B744" s="6" t="s">
+        <v>1463</v>
+      </c>
+      <c r="C744" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D744" s="14">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="745" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A745" s="1" t="s">
+        <v>1464</v>
+      </c>
+      <c r="B745" s="6" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C745" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D745" s="14">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="746" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A746" s="1" t="s">
+        <v>1466</v>
+      </c>
+      <c r="B746" s="6" t="s">
+        <v>1467</v>
+      </c>
+      <c r="C746" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D746" s="14">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="747" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A747" s="1" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B747" s="6" t="s">
+        <v>1469</v>
+      </c>
+      <c r="C747" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D747" s="14">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="748" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A748" s="1" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B748" s="6" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C748" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D748" s="14">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="749" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A749" s="1" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B749" s="6" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C749" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D749" s="14">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="750" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A750" s="1" t="s">
+        <v>1474</v>
+      </c>
+      <c r="B750" s="6" t="s">
+        <v>1475</v>
+      </c>
+      <c r="C750" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D750" s="14">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="751" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A751" s="1" t="s">
+        <v>1476</v>
+      </c>
+      <c r="B751" s="6" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C751" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D751" s="14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="752" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A752" s="1" t="s">
+        <v>1478</v>
+      </c>
+      <c r="B752" s="6" t="s">
+        <v>1479</v>
+      </c>
+      <c r="C752" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D752" s="14">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="753" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A753" s="1" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B753" s="6" t="s">
+        <v>1481</v>
+      </c>
+      <c r="C753" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D753" s="14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="754" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A754" s="1" t="s">
+        <v>1482</v>
+      </c>
+      <c r="B754" s="6" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C754" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D754" s="14">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="755" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A755" s="1" t="s">
+        <v>1484</v>
+      </c>
+      <c r="B755" s="6" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C755" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D755" s="14">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="756" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A756" s="1" t="s">
+        <v>1485</v>
+      </c>
+      <c r="B756" s="6" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C756" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D756" s="14">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="757" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A757" s="1" t="s">
+        <v>1487</v>
+      </c>
+      <c r="B757" s="6" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C757" s="13" t="s">
+        <v>521</v>
+      </c>
+      <c r="D757" s="14">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="758" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A758" s="1" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B758" s="6" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C758" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D758" s="14">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="759" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A759" s="1" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B759" s="6" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C759" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D759" s="14">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="760" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A760" s="1" t="s">
+        <v>1493</v>
+      </c>
+      <c r="B760" s="6" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C760" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D760" s="14">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="761" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A761" s="1" t="s">
+        <v>1495</v>
+      </c>
+      <c r="B761" s="6" t="s">
+        <v>1496</v>
+      </c>
+      <c r="C761" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D761" s="14">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="762" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A762" s="1" t="s">
+        <v>1497</v>
+      </c>
+      <c r="B762" s="6" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C762" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D762" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="763" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A763" s="1" t="s">
+        <v>1499</v>
+      </c>
+      <c r="B763" s="6" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C763" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D763" s="14">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="764" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A764" s="1" t="s">
+        <v>1501</v>
+      </c>
+      <c r="B764" s="6" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C764" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D764" s="14">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="765" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A765" s="1" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B765" s="6" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C765" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D765" s="14">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="766" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A766" s="1" t="s">
+        <v>1505</v>
+      </c>
+      <c r="B766" s="6" t="s">
+        <v>1506</v>
+      </c>
+      <c r="C766" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D766" s="14">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="767" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A767" s="7" t="s">
+        <v>1507</v>
+      </c>
+      <c r="B767" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C767" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D767" s="15">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="768" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A768" s="7" t="s">
+        <v>1508</v>
+      </c>
+      <c r="B768" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C768" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D768" s="15">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="769" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A769" s="7" t="s">
+        <v>1509</v>
+      </c>
+      <c r="B769" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C769" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D769" s="15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="770" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A770" s="7" t="s">
+        <v>1510</v>
+      </c>
+      <c r="B770" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C770" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D770" s="4">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="771" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A771" s="7" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B771" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C771" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D771" s="15">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="772" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A772" s="7" t="s">
+        <v>1512</v>
+      </c>
+      <c r="B772" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C772" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D772" s="4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="773" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A773" s="7" t="s">
+        <v>1513</v>
+      </c>
+      <c r="B773" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C773" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D773" s="15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="774" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A774" s="7" t="s">
+        <v>1514</v>
+      </c>
+      <c r="B774" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C774" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D774" s="15">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="775" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A775" s="7" t="s">
+        <v>1515</v>
+      </c>
+      <c r="B775" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C775" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D775" s="15">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="776" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A776" s="7" t="s">
+        <v>1516</v>
+      </c>
+      <c r="B776" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C776" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D776" s="15">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="777" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A777" s="7" t="s">
+        <v>1517</v>
+      </c>
+      <c r="B777" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C777" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D777" s="15">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="778" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A778" s="7" t="s">
+        <v>1518</v>
+      </c>
+      <c r="B778" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C778" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D778" s="16">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="779" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A779" s="7" t="s">
+        <v>1519</v>
+      </c>
+      <c r="B779" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C779" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D779" s="16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="780" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A780" s="7" t="s">
+        <v>1520</v>
+      </c>
+      <c r="B780" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C780" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D780" s="16">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="781" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A781" s="7" t="s">
+        <v>1521</v>
+      </c>
+      <c r="B781" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C781" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D781" s="16">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="782" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A782" s="7" t="s">
+        <v>1522</v>
+      </c>
+      <c r="B782" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C782" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D782" s="16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="783" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A783" s="7" t="s">
+        <v>1523</v>
+      </c>
+      <c r="B783" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C783" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D783" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="784" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A784" s="7" t="s">
+        <v>1524</v>
+      </c>
+      <c r="B784" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C784" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D784" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="785" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A785" s="7" t="s">
+        <v>1525</v>
+      </c>
+      <c r="B785" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C785" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D785" s="16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="786" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A786" s="7" t="s">
+        <v>1526</v>
+      </c>
+      <c r="B786" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C786" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D786" s="16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="787" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A787" s="7" t="s">
+        <v>1527</v>
+      </c>
+      <c r="B787" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C787" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D787" s="16">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="788" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A788" s="7" t="s">
+        <v>1528</v>
+      </c>
+      <c r="B788" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C788" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D788" s="16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="789" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A789" s="7" t="s">
+        <v>1529</v>
+      </c>
+      <c r="B789" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C789" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D789" s="16">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="790" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A790" s="7" t="s">
+        <v>1530</v>
+      </c>
+      <c r="B790" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C790" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D790" s="16">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="791" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A791" s="7" t="s">
+        <v>1531</v>
+      </c>
+      <c r="B791" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C791" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D791" s="16">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="792" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A792" s="7" t="s">
+        <v>1532</v>
+      </c>
+      <c r="B792" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C792" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D792" s="16">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="793" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A793" s="7" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B793" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C793" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D793" s="16">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="794" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A794" s="7" t="s">
+        <v>1534</v>
+      </c>
+      <c r="B794" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C794" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D794" s="16">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="795" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A795" s="7" t="s">
+        <v>1535</v>
+      </c>
+      <c r="B795" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C795" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D795" s="16">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="796" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A796" s="7" t="s">
+        <v>1536</v>
+      </c>
+      <c r="B796" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C796" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D796" s="16">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="797" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A797" s="7" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B797" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C797" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D797" s="4">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="798" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A798" s="7" t="s">
+        <v>1538</v>
+      </c>
+      <c r="B798" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C798" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D798" s="4">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="799" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A799" s="7" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B799" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C799" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D799" s="16">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="800" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A800" s="7" t="s">
+        <v>1540</v>
+      </c>
+      <c r="B800" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C800" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D800" s="16">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="801" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A801" s="7" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B801" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C801" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D801" s="16">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="802" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A802" s="7" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B802" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C802" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D802" s="16">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="803" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A803" s="7" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B803" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C803" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D803" s="16">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="804" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A804" s="7" t="s">
+        <v>1544</v>
+      </c>
+      <c r="B804" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C804" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D804" s="16">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="805" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A805" s="7" t="s">
+        <v>1545</v>
+      </c>
+      <c r="B805" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C805" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D805" s="16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="806" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A806" s="7" t="s">
+        <v>1546</v>
+      </c>
+      <c r="B806" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C806" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D806" s="16">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="807" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A807" s="7" t="s">
+        <v>1547</v>
+      </c>
+      <c r="B807" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C807" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D807" s="16">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="808" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A808" s="7" t="s">
+        <v>1548</v>
+      </c>
+      <c r="B808" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="C808" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D808" s="16">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="809" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A809" s="7" t="s">
+        <v>1549</v>
+      </c>
+      <c r="B809" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C809" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D809" s="16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="810" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A810" s="7" t="s">
+        <v>1550</v>
+      </c>
+      <c r="B810" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="C810" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D810" s="16">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="811" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A811" s="7" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B811" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C811" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D811" s="16">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="812" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A812" s="7" t="s">
+        <v>1552</v>
+      </c>
+      <c r="B812" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="C812" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D812" s="16">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="813" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A813" s="7" t="s">
+        <v>1553</v>
+      </c>
+      <c r="B813" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C813" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D813" s="16">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="814" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A814" s="7" t="s">
+        <v>1554</v>
+      </c>
+      <c r="B814" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="C814" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D814" s="16">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="815" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A815" s="7" t="s">
+        <v>1555</v>
+      </c>
+      <c r="B815" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="C815" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D815" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="816" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A816" s="7" t="s">
+        <v>1556</v>
+      </c>
+      <c r="B816" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="C816" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D816" s="16">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="817" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A817" s="7" t="s">
+        <v>1557</v>
+      </c>
+      <c r="B817" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="C817" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D817" s="16">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="818" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A818" s="7" t="s">
+        <v>1558</v>
+      </c>
+      <c r="B818" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="C818" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D818" s="16">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="819" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A819" s="7" t="s">
+        <v>1559</v>
+      </c>
+      <c r="B819" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="C819" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D819" s="16">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="820" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A820" s="7" t="s">
+        <v>1560</v>
+      </c>
+      <c r="B820" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C820" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D820" s="16">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="821" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A821" s="7" t="s">
+        <v>1561</v>
+      </c>
+      <c r="B821" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="C821" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D821" s="16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="822" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A822" s="7" t="s">
+        <v>1562</v>
+      </c>
+      <c r="B822" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="C822" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D822" s="16">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="823" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A823" s="7" t="s">
+        <v>1563</v>
+      </c>
+      <c r="B823" s="2" t="s">
+        <v>768</v>
+      </c>
+      <c r="C823" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D823" s="16">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="824" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A824" s="7" t="s">
+        <v>1564</v>
+      </c>
+      <c r="B824" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="C824" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D824" s="16">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="825" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A825" s="7" t="s">
+        <v>1565</v>
+      </c>
+      <c r="B825" s="2" t="s">
+        <v>776</v>
+      </c>
+      <c r="C825" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D825" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="826" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A826" s="7" t="s">
+        <v>1566</v>
+      </c>
+      <c r="B826" s="2" t="s">
+        <v>778</v>
+      </c>
+      <c r="C826" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D826" s="16">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="827" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A827" s="7" t="s">
+        <v>1567</v>
+      </c>
+      <c r="B827" s="2" t="s">
+        <v>780</v>
+      </c>
+      <c r="C827" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D827" s="16">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="828" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A828" s="7" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B828" s="2" t="s">
+        <v>949</v>
+      </c>
+      <c r="C828" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D828" s="16">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="829" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A829" s="7" t="s">
+        <v>1569</v>
+      </c>
+      <c r="B829" s="2" t="s">
+        <v>951</v>
+      </c>
+      <c r="C829" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D829" s="16">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="830" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A830" s="7" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B830" s="2" t="s">
+        <v>961</v>
+      </c>
+      <c r="C830" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D830" s="16">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="831" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A831" s="7" t="s">
+        <v>1571</v>
+      </c>
+      <c r="B831" s="2" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C831" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D831" s="16">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="832" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A832" s="7" t="s">
+        <v>1572</v>
+      </c>
+      <c r="B832" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C832" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D832" s="16">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="833" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A833" s="7" t="s">
+        <v>1573</v>
+      </c>
+      <c r="B833" s="2" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C833" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D833" s="16">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="834" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A834" s="7" t="s">
+        <v>1574</v>
+      </c>
+      <c r="B834" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C834" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D834" s="16">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="835" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A835" s="7" t="s">
+        <v>1575</v>
+      </c>
+      <c r="B835" s="2" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C835" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D835" s="16">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="836" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A836" s="7" t="s">
+        <v>1576</v>
+      </c>
+      <c r="B836" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C836" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D836" s="16">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="837" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A837" s="7" t="s">
+        <v>1577</v>
+      </c>
+      <c r="B837" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C837" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D837" s="16">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="838" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A838" s="7" t="s">
+        <v>1578</v>
+      </c>
+      <c r="B838" s="2" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C838" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D838" s="16">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="839" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A839" s="7" t="s">
+        <v>1579</v>
+      </c>
+      <c r="B839" s="2" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C839" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D839" s="16">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="840" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A840" s="7" t="s">
+        <v>1580</v>
+      </c>
+      <c r="B840" s="2" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C840" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D840" s="16">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="841" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A841" s="7" t="s">
+        <v>1581</v>
+      </c>
+      <c r="B841" s="2" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C841" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D841" s="16">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="842" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A842" s="7" t="s">
+        <v>1582</v>
+      </c>
+      <c r="B842" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C842" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D842" s="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="843" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A843" s="7" t="s">
+        <v>1583</v>
+      </c>
+      <c r="B843" s="2" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C843" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D843" s="16">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="844" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A844" s="7" t="s">
+        <v>1584</v>
+      </c>
+      <c r="B844" s="2" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C844" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D844" s="16">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="845" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A845" s="7" t="s">
+        <v>1585</v>
+      </c>
+      <c r="B845" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="C845" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D845" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="846" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A846" s="7" t="s">
+        <v>1586</v>
+      </c>
+      <c r="B846" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C846" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D846" s="16">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="847" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A847" s="7" t="s">
+        <v>1587</v>
+      </c>
+      <c r="B847" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="C847" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D847" s="16">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="848" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A848" s="7" t="s">
+        <v>1588</v>
+      </c>
+      <c r="B848" s="2" t="s">
+        <v>1209</v>
+      </c>
+      <c r="C848" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D848" s="16">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="849" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A849" s="7" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B849" s="2" t="s">
+        <v>1211</v>
+      </c>
+      <c r="C849" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D849" s="16">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="850" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A850" s="7" t="s">
+        <v>1590</v>
+      </c>
+      <c r="B850" s="2" t="s">
+        <v>1233</v>
+      </c>
+      <c r="C850" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D850" s="16">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="851" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A851" s="7" t="s">
+        <v>1591</v>
+      </c>
+      <c r="B851" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C851" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D851" s="16">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="852" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A852" s="7" t="s">
+        <v>1592</v>
+      </c>
+      <c r="B852" s="2" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C852" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D852" s="16">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="853" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A853" s="7" t="s">
+        <v>1593</v>
+      </c>
+      <c r="B853" s="2" t="s">
+        <v>1239</v>
+      </c>
+      <c r="C853" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D853" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="854" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A854" s="7" t="s">
+        <v>1594</v>
+      </c>
+      <c r="B854" s="2" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C854" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D854" s="16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="855" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A855" s="7" t="s">
+        <v>1595</v>
+      </c>
+      <c r="B855" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C855" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D855" s="16">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="856" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A856" s="7" t="s">
+        <v>1596</v>
+      </c>
+      <c r="B856" s="2" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C856" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D856" s="16">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="857" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A857" s="7" t="s">
+        <v>1597</v>
+      </c>
+      <c r="B857" s="2" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C857" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D857" s="16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="858" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A858" s="7" t="s">
+        <v>1598</v>
+      </c>
+      <c r="B858" s="2" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C858" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D858" s="16">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="859" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A859" s="7" t="s">
+        <v>1599</v>
+      </c>
+      <c r="B859" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C859" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D859" s="16">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="860" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A860" s="7" t="s">
+        <v>1600</v>
+      </c>
+      <c r="B860" s="2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C860" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D860" s="16">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="861" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A861" s="7" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B861" s="2" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C861" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D861" s="16">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="862" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A862" s="7" t="s">
+        <v>1602</v>
+      </c>
+      <c r="B862" s="2" t="s">
+        <v>1273</v>
+      </c>
+      <c r="C862" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D862" s="16">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="863" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A863" s="7" t="s">
+        <v>1603</v>
+      </c>
+      <c r="B863" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C863" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D863" s="16">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="864" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A864" s="7" t="s">
+        <v>1604</v>
+      </c>
+      <c r="B864" s="2" t="s">
+        <v>1605</v>
+      </c>
+      <c r="C864" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D864" s="16">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="865" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A865" s="7" t="s">
+        <v>1606</v>
+      </c>
+      <c r="B865" s="2" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C865" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D865" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="866" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A866" s="7" t="s">
+        <v>1608</v>
+      </c>
+      <c r="B866" s="2" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C866" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D866" s="16">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="867" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A867" s="7" t="s">
+        <v>1610</v>
+      </c>
+      <c r="B867" s="2" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C867" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D867" s="16">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="868" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A868" s="7" t="s">
+        <v>1612</v>
+      </c>
+      <c r="B868" s="2" t="s">
+        <v>1613</v>
+      </c>
+      <c r="C868" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D868" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="869" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A869" s="7" t="s">
+        <v>1614</v>
+      </c>
+      <c r="B869" s="2" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C869" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D869" s="16">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="870" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A870" s="7" t="s">
+        <v>1615</v>
+      </c>
+      <c r="B870" s="2" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C870" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D870" s="16">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="871" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A871" s="7" t="s">
+        <v>1616</v>
+      </c>
+      <c r="B871" s="2" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C871" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D871" s="16">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="872" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A872" s="7" t="s">
+        <v>1617</v>
+      </c>
+      <c r="B872" s="2" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C872" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D872" s="16">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="873" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A873" s="7" t="s">
+        <v>1618</v>
+      </c>
+      <c r="B873" s="2" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C873" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D873" s="16">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="874" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A874" s="7" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B874" s="2" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C874" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D874" s="16">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="875" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A875" s="7" t="s">
+        <v>1620</v>
+      </c>
+      <c r="B875" s="2" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C875" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D875" s="16">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="876" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A876" s="7" t="s">
+        <v>1621</v>
+      </c>
+      <c r="B876" s="2" t="s">
+        <v>1622</v>
+      </c>
+      <c r="C876" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D876" s="16">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="877" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A877" s="7" t="s">
+        <v>1623</v>
+      </c>
+      <c r="B877" s="2" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C877" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D877" s="16">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="878" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A878" s="7" t="s">
+        <v>1624</v>
+      </c>
+      <c r="B878" s="2" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C878" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D878" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="879" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A879" s="7" t="s">
+        <v>1625</v>
+      </c>
+      <c r="B879" s="2" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C879" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D879" s="16">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>